<commit_message>
identify the number of "correct" LCAs made by each model
</commit_message>
<xml_diff>
--- a/data/qa_dataset/results/ranking_mAP.xlsx
+++ b/data/qa_dataset/results/ranking_mAP.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\PycharmProjects\llm-goal-scope\data\qa_dataset\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF61DD43-227F-4A6D-8D65-DE553E6C0AC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6307CCF1-81A6-4385-831D-2707174C0F5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{D25027FC-FC27-47EF-8BDA-CB9196E400CB}"/>
+    <workbookView xWindow="2550" yWindow="2550" windowWidth="14745" windowHeight="13620" xr2:uid="{D25027FC-FC27-47EF-8BDA-CB9196E400CB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -226,7 +226,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -282,6 +282,33 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -292,36 +319,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -665,56 +662,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="19" t="s">
+      <c r="B1" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="21" t="s">
+      <c r="C1" s="30" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="23" t="s">
+      <c r="E1" s="26" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="23" t="s">
+      <c r="F1" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="23" t="s">
+      <c r="G1" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="23" t="s">
+      <c r="H1" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="23" t="s">
+      <c r="I1" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="23" t="s">
+      <c r="J1" s="26" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="20"/>
-      <c r="B2" s="20"/>
-      <c r="C2" s="22"/>
+      <c r="A2" s="29"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="31"/>
       <c r="D2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-      <c r="I2" s="24"/>
-      <c r="J2" s="24"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="27"/>
+      <c r="J2" s="27"/>
     </row>
     <row r="3" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="26" t="s">
+      <c r="A3" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="26" t="s">
+      <c r="B3" s="19" t="s">
         <v>12</v>
       </c>
       <c r="C3" s="1" t="s">
@@ -743,8 +740,8 @@
       </c>
     </row>
     <row r="4" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="25"/>
-      <c r="B4" s="25"/>
+      <c r="A4" s="20"/>
+      <c r="B4" s="20"/>
       <c r="C4" s="1" t="s">
         <v>14</v>
       </c>
@@ -771,8 +768,8 @@
       </c>
     </row>
     <row r="5" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="25"/>
-      <c r="B5" s="25"/>
+      <c r="A5" s="20"/>
+      <c r="B5" s="20"/>
       <c r="C5" s="1" t="s">
         <v>15</v>
       </c>
@@ -799,8 +796,8 @@
       </c>
     </row>
     <row r="6" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="25"/>
-      <c r="B6" s="28"/>
+      <c r="A6" s="20"/>
+      <c r="B6" s="22"/>
       <c r="C6" s="7" t="s">
         <v>16</v>
       </c>
@@ -827,8 +824,8 @@
       </c>
     </row>
     <row r="7" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="25"/>
-      <c r="B7" s="29" t="s">
+      <c r="A7" s="20"/>
+      <c r="B7" s="23" t="s">
         <v>17</v>
       </c>
       <c r="C7" s="1" t="s">
@@ -857,8 +854,8 @@
       </c>
     </row>
     <row r="8" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="25"/>
-      <c r="B8" s="25"/>
+      <c r="A8" s="20"/>
+      <c r="B8" s="20"/>
       <c r="C8" s="1" t="s">
         <v>14</v>
       </c>
@@ -885,8 +882,8 @@
       </c>
     </row>
     <row r="9" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="25"/>
-      <c r="B9" s="25"/>
+      <c r="A9" s="20"/>
+      <c r="B9" s="20"/>
       <c r="C9" s="1" t="s">
         <v>15</v>
       </c>
@@ -913,8 +910,8 @@
       </c>
     </row>
     <row r="10" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="27"/>
-      <c r="B10" s="27"/>
+      <c r="A10" s="21"/>
+      <c r="B10" s="21"/>
       <c r="C10" s="11" t="s">
         <v>16</v>
       </c>
@@ -941,10 +938,10 @@
       </c>
     </row>
     <row r="11" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="30" t="s">
+      <c r="A11" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="30" t="s">
+      <c r="B11" s="24" t="s">
         <v>12</v>
       </c>
       <c r="C11" s="1" t="s">
@@ -973,8 +970,8 @@
       </c>
     </row>
     <row r="12" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="25"/>
-      <c r="B12" s="25"/>
+      <c r="A12" s="20"/>
+      <c r="B12" s="20"/>
       <c r="C12" s="1" t="s">
         <v>15</v>
       </c>
@@ -1001,8 +998,8 @@
       </c>
     </row>
     <row r="13" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="25"/>
-      <c r="B13" s="28"/>
+      <c r="A13" s="20"/>
+      <c r="B13" s="22"/>
       <c r="C13" s="7" t="s">
         <v>16</v>
       </c>
@@ -1029,8 +1026,8 @@
       </c>
     </row>
     <row r="14" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="25"/>
-      <c r="B14" s="29" t="s">
+      <c r="A14" s="20"/>
+      <c r="B14" s="23" t="s">
         <v>17</v>
       </c>
       <c r="C14" s="1" t="s">
@@ -1059,8 +1056,8 @@
       </c>
     </row>
     <row r="15" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="25"/>
-      <c r="B15" s="25"/>
+      <c r="A15" s="20"/>
+      <c r="B15" s="20"/>
       <c r="C15" s="1" t="s">
         <v>15</v>
       </c>
@@ -1087,8 +1084,8 @@
       </c>
     </row>
     <row r="16" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="31"/>
-      <c r="B16" s="31"/>
+      <c r="A16" s="25"/>
+      <c r="B16" s="25"/>
       <c r="C16" s="15" t="s">
         <v>16</v>
       </c>
@@ -1116,555 +1113,555 @@
     </row>
     <row r="17" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="18" spans="1:10" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="19" t="s">
+      <c r="A18" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="B18" s="19" t="s">
+      <c r="B18" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="C18" s="21" t="s">
+      <c r="C18" s="30" t="s">
         <v>2</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E18" s="23" t="s">
+      <c r="E18" s="26" t="s">
         <v>5</v>
       </c>
-      <c r="F18" s="23" t="s">
+      <c r="F18" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="G18" s="23" t="s">
+      <c r="G18" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="H18" s="23" t="s">
+      <c r="H18" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="I18" s="23" t="s">
+      <c r="I18" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="J18" s="23" t="s">
+      <c r="J18" s="26" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="20"/>
-      <c r="B19" s="20"/>
-      <c r="C19" s="22"/>
+      <c r="A19" s="29"/>
+      <c r="B19" s="29"/>
+      <c r="C19" s="31"/>
       <c r="D19" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="E19" s="24"/>
-      <c r="F19" s="24"/>
-      <c r="G19" s="24"/>
-      <c r="H19" s="24"/>
-      <c r="I19" s="24"/>
-      <c r="J19" s="24"/>
+      <c r="E19" s="27"/>
+      <c r="F19" s="27"/>
+      <c r="G19" s="27"/>
+      <c r="H19" s="27"/>
+      <c r="I19" s="27"/>
+      <c r="J19" s="27"/>
     </row>
     <row r="20" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A20" s="26" t="s">
+      <c r="A20" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="B20" s="26" t="s">
+      <c r="B20" s="19" t="s">
         <v>12</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>13</v>
       </c>
       <c r="D20" s="2">
-        <f>_xlfn.RANK.AVG(D3, $D3:$J3, 0)</f>
+        <f t="shared" ref="D20:D33" si="0">_xlfn.RANK.AVG(D3, $D3:$J3, 0)</f>
         <v>4</v>
       </c>
       <c r="E20" s="2">
-        <f t="shared" ref="E20:J35" si="0">_xlfn.RANK.AVG(E3, $D3:$J3, 0)</f>
+        <f t="shared" ref="E20:J33" si="1">_xlfn.RANK.AVG(E3, $D3:$J3, 0)</f>
         <v>7</v>
       </c>
       <c r="F20" s="2">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="G20" s="2">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="H20" s="2">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="I20" s="2">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="J20" s="2">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A21" s="20"/>
+      <c r="B21" s="20"/>
+      <c r="C21" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D21" s="2">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="E21" s="2">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="F21" s="2">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="G21" s="2">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="H21" s="2">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="I21" s="2">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="J21" s="2">
+        <f t="shared" si="1"/>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A22" s="20"/>
+      <c r="B22" s="20"/>
+      <c r="C22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D22" s="2">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="E22" s="2">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="F22" s="2">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="G22" s="2">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="H22" s="2">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="I22" s="2">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="J22" s="2">
+        <f t="shared" si="1"/>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="20"/>
+      <c r="B23" s="22"/>
+      <c r="C23" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D23" s="2">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="E23" s="2">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="F23" s="2">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="G23" s="2">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="H23" s="2">
+        <f t="shared" si="1"/>
+        <v>7</v>
+      </c>
+      <c r="I23" s="2">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="J23" s="2">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A24" s="20"/>
+      <c r="B24" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D24" s="2">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="E24" s="2">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="F24" s="2">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="G24" s="2">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="H24" s="2">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="I24" s="2">
+        <f t="shared" si="1"/>
+        <v>7</v>
+      </c>
+      <c r="J24" s="2">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A25" s="20"/>
+      <c r="B25" s="20"/>
+      <c r="C25" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D25" s="2">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="G20" s="2">
+      <c r="E25" s="2">
+        <f t="shared" si="1"/>
+        <v>7</v>
+      </c>
+      <c r="F25" s="2">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="G25" s="2">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="H25" s="2">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="I25" s="2">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="J25" s="2">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A26" s="20"/>
+      <c r="B26" s="20"/>
+      <c r="C26" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D26" s="2">
         <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="E26" s="2">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="F26" s="2">
+        <f t="shared" si="1"/>
+        <v>7</v>
+      </c>
+      <c r="G26" s="2">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="H26" s="2">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="I26" s="2">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="J26" s="2">
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="H20" s="2">
+    </row>
+    <row r="27" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="21"/>
+      <c r="B27" s="21"/>
+      <c r="C27" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D27" s="2">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="E27" s="2">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="F27" s="2">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="G27" s="2">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="H27" s="2">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="I27" s="2">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="J27" s="2">
+        <f t="shared" si="1"/>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A28" s="24" t="s">
+        <v>18</v>
+      </c>
+      <c r="B28" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D28" s="2">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="I20" s="2">
+      <c r="E28" s="2">
+        <f t="shared" si="1"/>
+        <v>7</v>
+      </c>
+      <c r="F28" s="2">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="G28" s="2">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="H28" s="2">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="I28" s="2">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="J28" s="2">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A29" s="20"/>
+      <c r="B29" s="20"/>
+      <c r="C29" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D29" s="2">
+        <f t="shared" si="0"/>
+        <v>2.5</v>
+      </c>
+      <c r="E29" s="2">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="F29" s="2">
+        <f t="shared" si="1"/>
+        <v>2.5</v>
+      </c>
+      <c r="G29" s="2">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="H29" s="2">
+        <f t="shared" si="1"/>
+        <v>7</v>
+      </c>
+      <c r="I29" s="2">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="J29" s="2">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="20"/>
+      <c r="B30" s="22"/>
+      <c r="C30" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D30" s="2">
+        <f t="shared" si="0"/>
+        <v>6.5</v>
+      </c>
+      <c r="E30" s="2">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="F30" s="2">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="G30" s="2">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="H30" s="2">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="I30" s="2">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="J30" s="2">
+        <f t="shared" si="1"/>
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A31" s="20"/>
+      <c r="B31" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D31" s="2">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="E31" s="2">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="F31" s="2">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="G31" s="2">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="H31" s="2">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="I31" s="2">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="J31" s="2">
+        <f t="shared" si="1"/>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A32" s="20"/>
+      <c r="B32" s="20"/>
+      <c r="C32" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D32" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="E32" s="2">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="F32" s="2">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="G32" s="2">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="H32" s="2">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="I32" s="2">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="J32" s="2">
+        <f t="shared" si="1"/>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="25"/>
+      <c r="B33" s="25"/>
+      <c r="C33" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="D33" s="2">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="J20" s="2">
-        <f t="shared" si="0"/>
+      <c r="E33" s="2">
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
-    </row>
-    <row r="21" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A21" s="25"/>
-      <c r="B21" s="25"/>
-      <c r="C21" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D21" s="2">
-        <f>_xlfn.RANK.AVG(D4, $D4:$J4, 0)</f>
-        <v>2</v>
-      </c>
-      <c r="E21" s="2">
-        <f t="shared" si="0"/>
+      <c r="F33" s="2">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="G33" s="2">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="H33" s="2">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="I33" s="2">
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="F21" s="2">
-        <f t="shared" si="0"/>
-        <v>6</v>
-      </c>
-      <c r="G21" s="2">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="H21" s="2">
-        <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-      <c r="I21" s="2">
-        <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
-      <c r="J21" s="2">
-        <f t="shared" si="0"/>
+      <c r="J33" s="2">
+        <f t="shared" si="1"/>
         <v>7</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="25"/>
-      <c r="B22" s="25"/>
-      <c r="C22" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D22" s="2">
-        <f>_xlfn.RANK.AVG(D5, $D5:$J5, 0)</f>
-        <v>6</v>
-      </c>
-      <c r="E22" s="2">
-        <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-      <c r="F22" s="2">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="G22" s="2">
-        <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
-      <c r="H22" s="2">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="I22" s="2">
-        <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-      <c r="J22" s="2">
-        <f t="shared" si="0"/>
-        <v>7</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="25"/>
-      <c r="B23" s="28"/>
-      <c r="C23" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D23" s="2">
-        <f>_xlfn.RANK.AVG(D6, $D6:$J6, 0)</f>
-        <v>2</v>
-      </c>
-      <c r="E23" s="2">
-        <f t="shared" si="0"/>
-        <v>6</v>
-      </c>
-      <c r="F23" s="2">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="G23" s="2">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="H23" s="2">
-        <f t="shared" si="0"/>
-        <v>7</v>
-      </c>
-      <c r="I23" s="2">
-        <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
-      <c r="J23" s="2">
-        <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A24" s="25"/>
-      <c r="B24" s="29" t="s">
-        <v>17</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D24" s="2">
-        <f>_xlfn.RANK.AVG(D7, $D7:$J7, 0)</f>
-        <v>5</v>
-      </c>
-      <c r="E24" s="2">
-        <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
-      <c r="F24" s="2">
-        <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-      <c r="G24" s="2">
-        <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-      <c r="H24" s="2">
-        <f t="shared" si="0"/>
-        <v>6</v>
-      </c>
-      <c r="I24" s="2">
-        <f t="shared" si="0"/>
-        <v>7</v>
-      </c>
-      <c r="J24" s="2">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A25" s="25"/>
-      <c r="B25" s="25"/>
-      <c r="C25" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D25" s="2">
-        <f>_xlfn.RANK.AVG(D8, $D8:$J8, 0)</f>
-        <v>3</v>
-      </c>
-      <c r="E25" s="2">
-        <f t="shared" si="0"/>
-        <v>7</v>
-      </c>
-      <c r="F25" s="2">
-        <f t="shared" si="0"/>
-        <v>6</v>
-      </c>
-      <c r="G25" s="2">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="H25" s="2">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="I25" s="2">
-        <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
-      <c r="J25" s="2">
-        <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A26" s="25"/>
-      <c r="B26" s="25"/>
-      <c r="C26" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D26" s="2">
-        <f>_xlfn.RANK.AVG(D9, $D9:$J9, 0)</f>
-        <v>4</v>
-      </c>
-      <c r="E26" s="2">
-        <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-      <c r="F26" s="2">
-        <f t="shared" si="0"/>
-        <v>7</v>
-      </c>
-      <c r="G26" s="2">
-        <f t="shared" si="0"/>
-        <v>6</v>
-      </c>
-      <c r="H26" s="2">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="I26" s="2">
-        <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-      <c r="J26" s="2">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="27"/>
-      <c r="B27" s="27"/>
-      <c r="C27" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="D27" s="2">
-        <f>_xlfn.RANK.AVG(D10, $D10:$J10, 0)</f>
-        <v>4</v>
-      </c>
-      <c r="E27" s="2">
-        <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-      <c r="F27" s="2">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="G27" s="2">
-        <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-      <c r="H27" s="2">
-        <f t="shared" si="0"/>
-        <v>6</v>
-      </c>
-      <c r="I27" s="2">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J27" s="2">
-        <f t="shared" si="0"/>
-        <v>7</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A28" s="30" t="s">
-        <v>18</v>
-      </c>
-      <c r="B28" s="30" t="s">
-        <v>12</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D28" s="2">
-        <f>_xlfn.RANK.AVG(D11, $D11:$J11, 0)</f>
-        <v>1</v>
-      </c>
-      <c r="E28" s="2">
-        <f t="shared" si="0"/>
-        <v>7</v>
-      </c>
-      <c r="F28" s="2">
-        <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-      <c r="G28" s="2">
-        <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-      <c r="H28" s="2">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="I28" s="2">
-        <f t="shared" si="0"/>
-        <v>6</v>
-      </c>
-      <c r="J28" s="2">
-        <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A29" s="25"/>
-      <c r="B29" s="25"/>
-      <c r="C29" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D29" s="2">
-        <f>_xlfn.RANK.AVG(D12, $D12:$J12, 0)</f>
-        <v>2.5</v>
-      </c>
-      <c r="E29" s="2">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="F29" s="2">
-        <f t="shared" si="0"/>
-        <v>2.5</v>
-      </c>
-      <c r="G29" s="2">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="H29" s="2">
-        <f t="shared" si="0"/>
-        <v>7</v>
-      </c>
-      <c r="I29" s="2">
-        <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
-      <c r="J29" s="2">
-        <f t="shared" si="0"/>
-        <v>6</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="25"/>
-      <c r="B30" s="28"/>
-      <c r="C30" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D30" s="2">
-        <f>_xlfn.RANK.AVG(D13, $D13:$J13, 0)</f>
-        <v>6.5</v>
-      </c>
-      <c r="E30" s="2">
-        <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-      <c r="F30" s="2">
-        <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-      <c r="G30" s="2">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="H30" s="2">
-        <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
-      <c r="I30" s="2">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="J30" s="2">
-        <f t="shared" si="0"/>
-        <v>6.5</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A31" s="25"/>
-      <c r="B31" s="29" t="s">
-        <v>17</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D31" s="2">
-        <f>_xlfn.RANK.AVG(D14, $D14:$J14, 0)</f>
-        <v>2</v>
-      </c>
-      <c r="E31" s="2">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="F31" s="2">
-        <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
-      <c r="G31" s="2">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="H31" s="2">
-        <f t="shared" si="0"/>
-        <v>6</v>
-      </c>
-      <c r="I31" s="2">
-        <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-      <c r="J31" s="2">
-        <f t="shared" si="0"/>
-        <v>7</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A32" s="25"/>
-      <c r="B32" s="25"/>
-      <c r="C32" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D32" s="2">
-        <f>_xlfn.RANK.AVG(D15, $D15:$J15, 0)</f>
-        <v>3</v>
-      </c>
-      <c r="E32" s="2">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="F32" s="2">
-        <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
-      <c r="G32" s="2">
-        <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-      <c r="H32" s="2">
-        <f t="shared" si="0"/>
-        <v>6</v>
-      </c>
-      <c r="I32" s="2">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J32" s="2">
-        <f t="shared" si="0"/>
-        <v>7</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="31"/>
-      <c r="B33" s="31"/>
-      <c r="C33" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="D33" s="2">
-        <f>_xlfn.RANK.AVG(D16, $D16:$J16, 0)</f>
-        <v>6</v>
-      </c>
-      <c r="E33" s="2">
-        <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-      <c r="F33" s="2">
-        <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
-      <c r="G33" s="2">
-        <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-      <c r="H33" s="2">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="I33" s="2">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J33" s="2">
-        <f t="shared" si="0"/>
-        <v>7</v>
-      </c>
-    </row>
     <row r="34" spans="1:10" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="C34" s="32" t="s">
+      <c r="C34" s="1" t="s">
         <v>19</v>
       </c>
       <c r="D34" s="2">
@@ -1672,32 +1669,32 @@
         <v>3.6428571428571428</v>
       </c>
       <c r="E34" s="2">
-        <f t="shared" ref="E34:J34" si="1">AVERAGE(E20:E33)</f>
+        <f t="shared" ref="E34:J34" si="2">AVERAGE(E20:E33)</f>
         <v>4.0714285714285712</v>
       </c>
       <c r="F34" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4.1785714285714288</v>
       </c>
       <c r="G34" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.9285714285714284</v>
       </c>
       <c r="H34" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4.5</v>
       </c>
       <c r="I34" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3.5714285714285716</v>
       </c>
       <c r="J34" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>5.1071428571428568</v>
       </c>
     </row>
     <row r="35" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="C35" s="32" t="s">
+      <c r="C35" s="1" t="s">
         <v>20</v>
       </c>
       <c r="D35" s="2">
@@ -1705,50 +1702,32 @@
         <v>3</v>
       </c>
       <c r="E35" s="2">
-        <f t="shared" ref="E35:J35" si="2">_xlfn.RANK.AVG(E34, $D34:$J34, 1)</f>
+        <f t="shared" ref="E35:J35" si="3">_xlfn.RANK.AVG(E34, $D34:$J34, 1)</f>
         <v>4</v>
       </c>
       <c r="F35" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>5</v>
       </c>
       <c r="G35" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="H35" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>6</v>
       </c>
       <c r="I35" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>2</v>
       </c>
       <c r="J35" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>7</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="A20:A27"/>
-    <mergeCell ref="B20:B23"/>
-    <mergeCell ref="B24:B27"/>
-    <mergeCell ref="A28:A33"/>
-    <mergeCell ref="B28:B30"/>
-    <mergeCell ref="B31:B33"/>
-    <mergeCell ref="E18:E19"/>
-    <mergeCell ref="F18:F19"/>
-    <mergeCell ref="G18:G19"/>
-    <mergeCell ref="H18:H19"/>
-    <mergeCell ref="I18:I19"/>
-    <mergeCell ref="J18:J19"/>
-    <mergeCell ref="A11:A16"/>
-    <mergeCell ref="B11:B13"/>
-    <mergeCell ref="B14:B16"/>
-    <mergeCell ref="A18:A19"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="C18:C19"/>
     <mergeCell ref="H1:H2"/>
     <mergeCell ref="I1:I2"/>
     <mergeCell ref="J1:J2"/>
@@ -1761,6 +1740,24 @@
     <mergeCell ref="E1:E2"/>
     <mergeCell ref="F1:F2"/>
     <mergeCell ref="G1:G2"/>
+    <mergeCell ref="J18:J19"/>
+    <mergeCell ref="A11:A16"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="E18:E19"/>
+    <mergeCell ref="F18:F19"/>
+    <mergeCell ref="G18:G19"/>
+    <mergeCell ref="H18:H19"/>
+    <mergeCell ref="I18:I19"/>
+    <mergeCell ref="A20:A27"/>
+    <mergeCell ref="B20:B23"/>
+    <mergeCell ref="B24:B27"/>
+    <mergeCell ref="A28:A33"/>
+    <mergeCell ref="B28:B30"/>
+    <mergeCell ref="B31:B33"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
update label precision plots
</commit_message>
<xml_diff>
--- a/data/qa_dataset/results/ranking_mAP.xlsx
+++ b/data/qa_dataset/results/ranking_mAP.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\PycharmProjects\llm-goal-scope\data\qa_dataset\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{854A73AE-E077-4B45-BF97-5CBF7BBD0461}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D143D009-7002-447D-B116-D38BEB2A19BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{D25027FC-FC27-47EF-8BDA-CB9196E400CB}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="17385" xr2:uid="{D25027FC-FC27-47EF-8BDA-CB9196E400CB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="36">
   <si>
     <t>Dataset</t>
   </si>
@@ -123,12 +123,36 @@
   </si>
   <si>
     <t>Environmental-BERT-base</t>
+  </si>
+  <si>
+    <t>ESGBERT/EnvironmentalBERT-base</t>
+  </si>
+  <si>
+    <t>FacebookAI/roberta-large</t>
+  </si>
+  <si>
+    <t>climatebert/distilroberta-base-climate-f</t>
+  </si>
+  <si>
+    <t>google-bert/bert-base-uncased</t>
+  </si>
+  <si>
+    <t>microsoft/deberta-v3-base</t>
+  </si>
+  <si>
+    <t>microsoft/deberta-v3-large</t>
+  </si>
+  <si>
+    <t>microsoft/deberta-v3-small</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="166" formatCode="0.0000"/>
+  </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -306,51 +330,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -358,6 +337,49 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -702,64 +724,76 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:27" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="26" t="s">
+      <c r="B1" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="35" t="s">
+      <c r="C1" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E1" s="35" t="s">
-        <v>5</v>
-      </c>
-      <c r="F1" s="35" t="s">
-        <v>6</v>
-      </c>
-      <c r="G1" s="35" t="s">
-        <v>7</v>
-      </c>
-      <c r="H1" s="35" t="s">
-        <v>8</v>
-      </c>
-      <c r="I1" s="35" t="s">
-        <v>9</v>
-      </c>
-      <c r="J1" s="35" t="s">
-        <v>10</v>
-      </c>
-      <c r="K1" s="33"/>
+      <c r="D1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G1" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I1" t="s">
+        <v>34</v>
+      </c>
+      <c r="J1" t="s">
+        <v>35</v>
+      </c>
+      <c r="K1" s="2"/>
       <c r="R1" t="s">
         <v>22</v>
       </c>
-      <c r="W1" s="26" t="s">
+      <c r="W1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="X1" s="26" t="s">
+      <c r="X1" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="Y1" s="28" t="s">
+      <c r="Y1" s="29" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:27" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="27"/>
-      <c r="B2" s="27"/>
-      <c r="C2" s="36"/>
-      <c r="D2" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
-      <c r="G2" s="36"/>
-      <c r="H2" s="36"/>
-      <c r="I2" s="36"/>
-      <c r="J2" s="36"/>
-      <c r="K2" s="33"/>
+      <c r="A2" s="28"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="21"/>
+      <c r="D2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F2" t="s">
+        <v>31</v>
+      </c>
+      <c r="G2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J2" t="s">
+        <v>35</v>
+      </c>
+      <c r="K2" s="2"/>
       <c r="N2" t="s">
         <v>21</v>
       </c>
@@ -769,9 +803,9 @@
       <c r="R2" t="s">
         <v>23</v>
       </c>
-      <c r="W2" s="27"/>
-      <c r="X2" s="27"/>
-      <c r="Y2" s="29"/>
+      <c r="W2" s="28"/>
+      <c r="X2" s="28"/>
+      <c r="Y2" s="30"/>
       <c r="Z2" t="s">
         <v>27</v>
       </c>
@@ -780,62 +814,62 @@
       </c>
     </row>
     <row r="3" spans="1:27" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="21" t="s">
+      <c r="A3" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="21" t="s">
+      <c r="B3" s="31" t="s">
         <v>12</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="2">
-        <v>0.82620000000000005</v>
-      </c>
-      <c r="E3" s="2">
-        <v>0.62390000000000001</v>
-      </c>
-      <c r="F3" s="2">
-        <v>0.86839999999999995</v>
-      </c>
-      <c r="G3" s="2">
-        <v>0.76580000000000004</v>
-      </c>
-      <c r="H3" s="5">
-        <v>0.95050000000000001</v>
-      </c>
-      <c r="I3" s="2">
-        <v>0.70630000000000004</v>
-      </c>
-      <c r="J3" s="6">
-        <v>0.88429999999999997</v>
+      <c r="D3" s="36">
+        <v>0.78060871876661297</v>
+      </c>
+      <c r="E3" s="36">
+        <v>0.58300264550264502</v>
+      </c>
+      <c r="F3" s="36">
+        <v>0.804593070104754</v>
+      </c>
+      <c r="G3" s="36">
+        <v>0.70246422893481697</v>
+      </c>
+      <c r="H3" s="36">
+        <v>0.822072072072072</v>
+      </c>
+      <c r="I3" s="36">
+        <v>0.65131578947368396</v>
+      </c>
+      <c r="J3" s="36">
+        <v>0.79793828697938196</v>
       </c>
       <c r="K3" s="6"/>
-      <c r="M3" s="32" t="s">
+      <c r="M3" s="35" t="s">
         <v>11</v>
       </c>
       <c r="N3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O3" s="34">
+      <c r="O3" s="19">
         <f>_xlfn.T.TEST(D3:J3,D7:J7,2,1)</f>
-        <v>0.23645553940447414</v>
-      </c>
-      <c r="Q3" s="32" t="s">
+        <v>0.22361051900129461</v>
+      </c>
+      <c r="Q3" s="35" t="s">
         <v>24</v>
       </c>
       <c r="R3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="T3" s="34">
+      <c r="T3" s="19">
         <f>_xlfn.T.TEST(D4:J4,D11:J11,2,1)</f>
-        <v>2.1333872228144991E-3</v>
-      </c>
-      <c r="V3" s="32"/>
-      <c r="W3" s="21" t="s">
+        <v>2.7364997224834504E-2</v>
+      </c>
+      <c r="V3" s="35"/>
+      <c r="W3" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="X3" s="21" t="s">
+      <c r="X3" s="31" t="s">
         <v>12</v>
       </c>
       <c r="Y3" s="1" t="s">
@@ -843,237 +877,237 @@
       </c>
       <c r="Z3">
         <f>MAX(D3:J3)</f>
-        <v>0.95050000000000001</v>
-      </c>
-      <c r="AA3" s="35" t="s">
+        <v>0.822072072072072</v>
+      </c>
+      <c r="AA3" s="20" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:27" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="22"/>
-      <c r="B4" s="22"/>
+      <c r="A4" s="23"/>
+      <c r="B4" s="23"/>
       <c r="C4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="6">
-        <v>0.78129999999999999</v>
-      </c>
-      <c r="E4" s="5">
-        <v>0.7994</v>
-      </c>
-      <c r="F4" s="2">
-        <v>0.6764</v>
-      </c>
-      <c r="G4" s="2">
-        <v>0.72389999999999999</v>
-      </c>
-      <c r="H4" s="2">
-        <v>0.76729999999999998</v>
-      </c>
-      <c r="I4" s="2">
-        <v>0.76390000000000002</v>
-      </c>
-      <c r="J4" s="2">
-        <v>0.63039999999999996</v>
+      <c r="D4" s="36">
+        <v>0.61399931473219804</v>
+      </c>
+      <c r="E4" s="36">
+        <v>0.62939369296105496</v>
+      </c>
+      <c r="F4" s="36">
+        <v>0.55447800271088599</v>
+      </c>
+      <c r="G4" s="36">
+        <v>0.60237628384687203</v>
+      </c>
+      <c r="H4" s="36">
+        <v>0.58621226268285098</v>
+      </c>
+      <c r="I4" s="36">
+        <v>0.61350659618686099</v>
+      </c>
+      <c r="J4" s="36">
+        <v>0.51599384973171303</v>
       </c>
       <c r="K4" s="2"/>
-      <c r="M4" s="32"/>
+      <c r="M4" s="35"/>
       <c r="N4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="O4" s="34">
-        <f t="shared" ref="O4:O9" si="0">_xlfn.T.TEST(D4:J4,D8:J8,2,1)</f>
-        <v>0.99705278858050428</v>
-      </c>
-      <c r="Q4" s="32"/>
+      <c r="O4" s="19">
+        <f t="shared" ref="O4:O6" si="0">_xlfn.T.TEST(D4:J4,D8:J8,2,1)</f>
+        <v>0.56216013992292602</v>
+      </c>
+      <c r="Q4" s="35"/>
       <c r="R4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="T4" s="34">
+      <c r="T4" s="19">
         <f>_xlfn.T.TEST(D5:J5,D12:J12,2,1)</f>
-        <v>6.3516894554757619E-4</v>
-      </c>
-      <c r="V4" s="32"/>
-      <c r="W4" s="22"/>
-      <c r="X4" s="22"/>
+        <v>2.48412124166407E-6</v>
+      </c>
+      <c r="V4" s="35"/>
+      <c r="W4" s="23"/>
+      <c r="X4" s="23"/>
       <c r="Y4" s="1" t="s">
         <v>14</v>
       </c>
       <c r="Z4">
         <f t="shared" ref="Z4:Z16" si="1">MAX(D4:J4)</f>
-        <v>0.7994</v>
-      </c>
-      <c r="AA4" s="35" t="s">
+        <v>0.62939369296105496</v>
+      </c>
+      <c r="AA4" s="20" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:27" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="22"/>
-      <c r="B5" s="22"/>
+      <c r="A5" s="23"/>
+      <c r="B5" s="23"/>
       <c r="C5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="2">
-        <v>0.87849999999999995</v>
-      </c>
-      <c r="E5" s="2">
-        <v>0.8841</v>
-      </c>
-      <c r="F5" s="2">
-        <v>0.87990000000000002</v>
-      </c>
-      <c r="G5" s="2">
-        <v>0.88129999999999997</v>
-      </c>
-      <c r="H5" s="5">
-        <v>0.89080000000000004</v>
-      </c>
-      <c r="I5" s="6">
-        <v>0.88649999999999995</v>
-      </c>
-      <c r="J5" s="2">
-        <v>0.87080000000000002</v>
+      <c r="D5" s="36">
+        <v>0.51472222222222197</v>
+      </c>
+      <c r="E5" s="36">
+        <v>0.51805555555555505</v>
+      </c>
+      <c r="F5" s="36">
+        <v>0.51555555555555499</v>
+      </c>
+      <c r="G5" s="36">
+        <v>0.51638888888888801</v>
+      </c>
+      <c r="H5" s="36">
+        <v>0.52194444444444399</v>
+      </c>
+      <c r="I5" s="36">
+        <v>0.51944444444444404</v>
+      </c>
+      <c r="J5" s="36">
+        <v>0.51022222222222202</v>
       </c>
       <c r="K5" s="2"/>
-      <c r="M5" s="32"/>
+      <c r="M5" s="35"/>
       <c r="N5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="O5" s="34">
+      <c r="O5" s="19">
         <f>_xlfn.T.TEST(D5:J5,D9:J9,2,1)</f>
-        <v>4.468426856691015E-2</v>
-      </c>
-      <c r="Q5" s="32"/>
+        <v>4.4812269605668378E-2</v>
+      </c>
+      <c r="Q5" s="35"/>
       <c r="R5" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="T5" s="34">
+      <c r="T5" s="19">
         <f>_xlfn.T.TEST(D6:J6,D13:J13,2,1)</f>
-        <v>2.0703782093450331E-2</v>
-      </c>
-      <c r="V5" s="32"/>
-      <c r="W5" s="22"/>
-      <c r="X5" s="22"/>
+        <v>1.8757927132676169E-2</v>
+      </c>
+      <c r="V5" s="35"/>
+      <c r="W5" s="23"/>
+      <c r="X5" s="23"/>
       <c r="Y5" s="1" t="s">
         <v>15</v>
       </c>
       <c r="Z5">
         <f t="shared" si="1"/>
-        <v>0.89080000000000004</v>
-      </c>
-      <c r="AA5" s="35" t="s">
+        <v>0.52194444444444399</v>
+      </c>
+      <c r="AA5" s="20" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:27" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="22"/>
+      <c r="A6" s="23"/>
       <c r="B6" s="24"/>
       <c r="C6" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="8">
-        <v>0.95620000000000005</v>
-      </c>
-      <c r="E6" s="9">
-        <v>0.93569999999999998</v>
-      </c>
-      <c r="F6" s="9">
-        <v>0.93979999999999997</v>
-      </c>
-      <c r="G6" s="10">
-        <v>0.96650000000000003</v>
-      </c>
-      <c r="H6" s="9">
-        <v>0.91479999999999995</v>
-      </c>
-      <c r="I6" s="9">
-        <v>0.94159999999999999</v>
-      </c>
-      <c r="J6" s="9">
-        <v>0.94199999999999995</v>
-      </c>
-      <c r="K6" s="33"/>
-      <c r="M6" s="32"/>
+      <c r="D6" s="36">
+        <v>0.97477685444490803</v>
+      </c>
+      <c r="E6" s="36">
+        <v>0.94501955544642302</v>
+      </c>
+      <c r="F6" s="36">
+        <v>0.94534569209015995</v>
+      </c>
+      <c r="G6" s="36">
+        <v>0.96911734238066005</v>
+      </c>
+      <c r="H6" s="36">
+        <v>0.93152219423916904</v>
+      </c>
+      <c r="I6" s="36">
+        <v>0.95446660958732699</v>
+      </c>
+      <c r="J6" s="36">
+        <v>0.94679965915643804</v>
+      </c>
+      <c r="K6" s="2"/>
+      <c r="M6" s="35"/>
       <c r="N6" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="O6" s="34">
+      <c r="O6" s="19">
         <f t="shared" si="0"/>
-        <v>0.17688730642356765</v>
-      </c>
-      <c r="Q6" s="32" t="s">
+        <v>0.2737058712852562</v>
+      </c>
+      <c r="Q6" s="35" t="s">
         <v>1</v>
       </c>
       <c r="R6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="T6" s="34">
+      <c r="T6" s="19">
         <f>_xlfn.T.TEST(D8:J8,D14:J14,2,1)</f>
-        <v>9.9465166096053229E-2</v>
-      </c>
-      <c r="V6" s="32"/>
-      <c r="W6" s="22"/>
+        <v>0.83972429370163293</v>
+      </c>
+      <c r="V6" s="35"/>
+      <c r="W6" s="23"/>
       <c r="X6" s="24"/>
       <c r="Y6" s="7" t="s">
         <v>16</v>
       </c>
       <c r="Z6">
         <f t="shared" si="1"/>
-        <v>0.96650000000000003</v>
-      </c>
-      <c r="AA6" s="35" t="s">
+        <v>0.97477685444490803</v>
+      </c>
+      <c r="AA6" s="20" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:27" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="22"/>
+      <c r="A7" s="23"/>
       <c r="B7" s="25" t="s">
         <v>17</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="2">
-        <v>0.75409999999999999</v>
-      </c>
-      <c r="E7" s="2">
-        <v>0.75519999999999998</v>
-      </c>
-      <c r="F7" s="2">
-        <v>0.76249999999999996</v>
-      </c>
-      <c r="G7" s="6">
-        <v>0.86209999999999998</v>
-      </c>
-      <c r="H7" s="2">
-        <v>0.63539999999999996</v>
-      </c>
-      <c r="I7" s="2">
-        <v>0.2</v>
-      </c>
-      <c r="J7" s="5">
-        <v>0.86560000000000004</v>
+      <c r="D7" s="36">
+        <v>0.67620160267219098</v>
+      </c>
+      <c r="E7" s="36">
+        <v>0.70097908913698304</v>
+      </c>
+      <c r="F7" s="36">
+        <v>0.69777777777777705</v>
+      </c>
+      <c r="G7" s="36">
+        <v>0.79837461300309498</v>
+      </c>
+      <c r="H7" s="36">
+        <v>0.59746212121212094</v>
+      </c>
+      <c r="I7" s="36">
+        <v>0.110576923076923</v>
+      </c>
+      <c r="J7" s="36">
+        <v>0.76025132275132201</v>
       </c>
       <c r="K7" s="5"/>
-      <c r="M7" s="32" t="s">
+      <c r="M7" s="35" t="s">
         <v>18</v>
       </c>
       <c r="N7" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="O7" s="34">
+      <c r="O7" s="19">
         <f>_xlfn.T.TEST(D11:J11,D14:J14,2,1)</f>
-        <v>2.5170554111090993E-3</v>
-      </c>
-      <c r="Q7" s="32"/>
+        <v>6.6932394955836636E-3</v>
+      </c>
+      <c r="Q7" s="35"/>
       <c r="R7" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="T7" s="34">
+      <c r="T7" s="19">
         <f t="shared" ref="T7:T8" si="2">_xlfn.T.TEST(D9:J9,D15:J15,2,1)</f>
-        <v>3.7346325711196603E-4</v>
-      </c>
-      <c r="W7" s="22"/>
+        <v>2.4684695804556842E-6</v>
+      </c>
+      <c r="W7" s="23"/>
       <c r="X7" s="25" t="s">
         <v>17</v>
       </c>
@@ -1082,195 +1116,195 @@
       </c>
       <c r="Z7">
         <f t="shared" si="1"/>
-        <v>0.86560000000000004</v>
-      </c>
-      <c r="AA7" s="35" t="s">
+        <v>0.79837461300309498</v>
+      </c>
+      <c r="AA7" s="20" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:27" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="22"/>
-      <c r="B8" s="22"/>
+      <c r="A8" s="23"/>
+      <c r="B8" s="23"/>
       <c r="C8" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="2">
-        <v>0.77480000000000004</v>
-      </c>
-      <c r="E8" s="2">
-        <v>0.6613</v>
-      </c>
-      <c r="F8" s="2">
-        <v>0.67510000000000003</v>
-      </c>
-      <c r="G8" s="5">
-        <v>0.79649999999999999</v>
-      </c>
-      <c r="H8" s="2">
-        <v>0.69189999999999996</v>
-      </c>
-      <c r="I8" s="2">
-        <v>0.74780000000000002</v>
-      </c>
-      <c r="J8" s="6">
-        <v>0.79620000000000002</v>
+      <c r="D8" s="36">
+        <v>0.60753871455462305</v>
+      </c>
+      <c r="E8" s="36">
+        <v>0.53450155730192095</v>
+      </c>
+      <c r="F8" s="36">
+        <v>0.53108362107148499</v>
+      </c>
+      <c r="G8" s="36">
+        <v>0.61772502268789697</v>
+      </c>
+      <c r="H8" s="36">
+        <v>0.544195848156244</v>
+      </c>
+      <c r="I8" s="36">
+        <v>0.57252238295848801</v>
+      </c>
+      <c r="J8" s="36">
+        <v>0.61200956244566795</v>
       </c>
       <c r="K8" s="6"/>
-      <c r="M8" s="32"/>
+      <c r="M8" s="35"/>
       <c r="N8" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="O8" s="34">
+      <c r="O8" s="19">
         <f t="shared" ref="O8:O9" si="3">_xlfn.T.TEST(D12:J12,D15:J15,2,1)</f>
-        <v>0.97853221978269223</v>
-      </c>
-      <c r="Q8" s="32"/>
+        <v>0.97579504118008287</v>
+      </c>
+      <c r="Q8" s="35"/>
       <c r="R8" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="T8" s="34">
+      <c r="T8" s="19">
         <f t="shared" si="2"/>
-        <v>5.4838243047406754E-3</v>
-      </c>
-      <c r="W8" s="22"/>
-      <c r="X8" s="22"/>
+        <v>3.3807876781668952E-2</v>
+      </c>
+      <c r="W8" s="23"/>
+      <c r="X8" s="23"/>
       <c r="Y8" s="1" t="s">
         <v>14</v>
       </c>
       <c r="Z8">
         <f t="shared" si="1"/>
-        <v>0.79649999999999999</v>
-      </c>
-      <c r="AA8" s="35" t="s">
+        <v>0.61772502268789697</v>
+      </c>
+      <c r="AA8" s="20" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:27" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="22"/>
-      <c r="B9" s="22"/>
+      <c r="A9" s="23"/>
+      <c r="B9" s="23"/>
       <c r="C9" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="2">
-        <v>0.87219999999999998</v>
-      </c>
-      <c r="E9" s="2">
-        <v>0.87360000000000004</v>
-      </c>
-      <c r="F9" s="2">
-        <v>0.85119999999999996</v>
-      </c>
-      <c r="G9" s="2">
-        <v>0.85850000000000004</v>
-      </c>
-      <c r="H9" s="5">
-        <v>0.89359999999999995</v>
-      </c>
-      <c r="I9" s="6">
-        <v>0.88370000000000004</v>
-      </c>
-      <c r="J9" s="2">
-        <v>0.86419999999999997</v>
+      <c r="D9" s="36">
+        <v>0.51105555555555504</v>
+      </c>
+      <c r="E9" s="36">
+        <v>0.51188888888888895</v>
+      </c>
+      <c r="F9" s="36">
+        <v>0.49870689655172401</v>
+      </c>
+      <c r="G9" s="36">
+        <v>0.503</v>
+      </c>
+      <c r="H9" s="36">
+        <v>0.52361111111111103</v>
+      </c>
+      <c r="I9" s="36">
+        <v>0.517777777777777</v>
+      </c>
+      <c r="J9" s="36">
+        <v>0.50633333333333297</v>
       </c>
       <c r="K9" s="2"/>
-      <c r="M9" s="32"/>
+      <c r="M9" s="35"/>
       <c r="N9" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="O9" s="34">
+      <c r="O9" s="19">
         <f t="shared" si="3"/>
-        <v>0.76270447665637353</v>
-      </c>
-      <c r="W9" s="22"/>
-      <c r="X9" s="22"/>
+        <v>0.78571786436059654</v>
+      </c>
+      <c r="W9" s="23"/>
+      <c r="X9" s="23"/>
       <c r="Y9" s="1" t="s">
         <v>15</v>
       </c>
       <c r="Z9">
         <f t="shared" si="1"/>
-        <v>0.89359999999999995</v>
-      </c>
-      <c r="AA9" s="35" t="s">
+        <v>0.52361111111111103</v>
+      </c>
+      <c r="AA9" s="20" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:27" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="23"/>
-      <c r="B10" s="23"/>
+      <c r="A10" s="32"/>
+      <c r="B10" s="32"/>
       <c r="C10" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="D10" s="12">
-        <v>0.93210000000000004</v>
-      </c>
-      <c r="E10" s="12">
-        <v>0.94499999999999995</v>
-      </c>
-      <c r="F10" s="12">
-        <v>0.90900000000000003</v>
-      </c>
-      <c r="G10" s="13">
-        <v>0.95030000000000003</v>
-      </c>
-      <c r="H10" s="12">
-        <v>0.89259999999999995</v>
-      </c>
-      <c r="I10" s="14">
-        <v>0.96850000000000003</v>
-      </c>
-      <c r="J10" s="12">
-        <v>0.85870000000000002</v>
-      </c>
-      <c r="K10" s="33"/>
-      <c r="W10" s="23"/>
-      <c r="X10" s="23"/>
+      <c r="D10" s="36">
+        <v>0.94657742209679596</v>
+      </c>
+      <c r="E10" s="36">
+        <v>0.96316154924443398</v>
+      </c>
+      <c r="F10" s="36">
+        <v>0.93226904503487396</v>
+      </c>
+      <c r="G10" s="36">
+        <v>0.95588696587349797</v>
+      </c>
+      <c r="H10" s="36">
+        <v>0.91574002165593205</v>
+      </c>
+      <c r="I10" s="36">
+        <v>0.97579114891973695</v>
+      </c>
+      <c r="J10" s="36">
+        <v>0.90263428562341297</v>
+      </c>
+      <c r="K10" s="2"/>
+      <c r="W10" s="32"/>
+      <c r="X10" s="32"/>
       <c r="Y10" s="11" t="s">
         <v>16</v>
       </c>
       <c r="Z10">
         <f t="shared" si="1"/>
-        <v>0.96850000000000003</v>
-      </c>
-      <c r="AA10" s="35" t="s">
+        <v>0.97579114891973695</v>
+      </c>
+      <c r="AA10" s="20" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:27" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="30" t="s">
+      <c r="A11" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="30" t="s">
+      <c r="B11" s="22" t="s">
         <v>12</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D11" s="5">
-        <v>0.90549999999999997</v>
-      </c>
-      <c r="E11" s="2">
-        <v>0.83040000000000003</v>
-      </c>
-      <c r="F11" s="2">
-        <v>0.90400000000000003</v>
-      </c>
-      <c r="G11" s="2">
-        <v>0.89410000000000001</v>
-      </c>
-      <c r="H11" s="2">
-        <v>0.88949999999999996</v>
-      </c>
-      <c r="I11" s="2">
-        <v>0.87629999999999997</v>
-      </c>
-      <c r="J11" s="2">
-        <v>0.89070000000000005</v>
+      <c r="D11" s="36">
+        <v>0.65436354869816704</v>
+      </c>
+      <c r="E11" s="36">
+        <v>0.606339869281045</v>
+      </c>
+      <c r="F11" s="36">
+        <v>0.66059139784946197</v>
+      </c>
+      <c r="G11" s="36">
+        <v>0.65501792114695301</v>
+      </c>
+      <c r="H11" s="36">
+        <v>0.65606605765874104</v>
+      </c>
+      <c r="I11" s="36">
+        <v>0.63836917562724005</v>
+      </c>
+      <c r="J11" s="36">
+        <v>0.65630402698713897</v>
       </c>
       <c r="K11" s="2"/>
-      <c r="W11" s="30" t="s">
+      <c r="W11" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="X11" s="30" t="s">
+      <c r="X11" s="22" t="s">
         <v>12</v>
       </c>
       <c r="Y11" s="1" t="s">
@@ -1278,125 +1312,125 @@
       </c>
       <c r="Z11">
         <f t="shared" si="1"/>
-        <v>0.90549999999999997</v>
+        <v>0.66059139784946197</v>
       </c>
       <c r="AA11" s="3" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:27" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="22"/>
-      <c r="B12" s="22"/>
+      <c r="A12" s="23"/>
+      <c r="B12" s="23"/>
       <c r="C12" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D12" s="6">
-        <v>0.95430000000000004</v>
-      </c>
-      <c r="E12" s="5">
-        <v>0.95740000000000003</v>
-      </c>
-      <c r="F12" s="6">
-        <v>0.95430000000000004</v>
-      </c>
-      <c r="G12" s="2">
-        <v>0.94620000000000004</v>
-      </c>
-      <c r="H12" s="2">
-        <v>0.8992</v>
-      </c>
-      <c r="I12" s="2">
-        <v>0.94799999999999995</v>
-      </c>
-      <c r="J12" s="2">
-        <v>0.92120000000000002</v>
+      <c r="D12" s="36">
+        <v>0.62653061224489803</v>
+      </c>
+      <c r="E12" s="36">
+        <v>0.628571428571428</v>
+      </c>
+      <c r="F12" s="36">
+        <v>0.62653061224489803</v>
+      </c>
+      <c r="G12" s="36">
+        <v>0.62121925693354196</v>
+      </c>
+      <c r="H12" s="36">
+        <v>0.59020408163265303</v>
+      </c>
+      <c r="I12" s="36">
+        <v>0.62240973312401804</v>
+      </c>
+      <c r="J12" s="36">
+        <v>0.60476190476190395</v>
       </c>
       <c r="K12" s="2"/>
-      <c r="W12" s="22"/>
-      <c r="X12" s="22"/>
+      <c r="W12" s="23"/>
+      <c r="X12" s="23"/>
       <c r="Y12" s="1" t="s">
         <v>15</v>
       </c>
       <c r="Z12">
         <f t="shared" si="1"/>
-        <v>0.95740000000000003</v>
-      </c>
-      <c r="AA12" s="35" t="s">
+        <v>0.628571428571428</v>
+      </c>
+      <c r="AA12" s="20" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:27" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="22"/>
+      <c r="A13" s="23"/>
       <c r="B13" s="24"/>
       <c r="C13" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D13" s="9">
-        <v>0.95130000000000003</v>
-      </c>
-      <c r="E13" s="9">
-        <v>0.97609999999999997</v>
-      </c>
-      <c r="F13" s="8">
-        <v>0.97760000000000002</v>
-      </c>
-      <c r="G13" s="10">
-        <v>0.98129999999999995</v>
-      </c>
-      <c r="H13" s="9">
-        <v>0.97529999999999994</v>
-      </c>
-      <c r="I13" s="9">
-        <v>0.96499999999999997</v>
-      </c>
-      <c r="J13" s="9">
-        <v>0.95130000000000003</v>
-      </c>
-      <c r="K13" s="33"/>
-      <c r="W13" s="22"/>
+      <c r="D13" s="36">
+        <v>0.90712999455402299</v>
+      </c>
+      <c r="E13" s="36">
+        <v>0.93978979951244701</v>
+      </c>
+      <c r="F13" s="36">
+        <v>0.93205711416606396</v>
+      </c>
+      <c r="G13" s="36">
+        <v>0.93662322338400295</v>
+      </c>
+      <c r="H13" s="36">
+        <v>0.92990370213885798</v>
+      </c>
+      <c r="I13" s="36">
+        <v>0.92009198843704199</v>
+      </c>
+      <c r="J13" s="36">
+        <v>0.90123963795217399</v>
+      </c>
+      <c r="K13" s="2"/>
+      <c r="W13" s="23"/>
       <c r="X13" s="24"/>
       <c r="Y13" s="7" t="s">
         <v>16</v>
       </c>
       <c r="Z13">
         <f t="shared" si="1"/>
-        <v>0.98129999999999995</v>
-      </c>
-      <c r="AA13" s="35" t="s">
+        <v>0.93978979951244701</v>
+      </c>
+      <c r="AA13" s="20" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="14" spans="1:27" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="22"/>
+      <c r="A14" s="23"/>
       <c r="B14" s="25" t="s">
         <v>17</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D14" s="6">
-        <v>0.8347</v>
-      </c>
-      <c r="E14" s="2">
-        <v>0.74150000000000005</v>
-      </c>
-      <c r="F14" s="2">
-        <v>0.78469999999999995</v>
-      </c>
-      <c r="G14" s="5">
-        <v>0.84719999999999995</v>
-      </c>
-      <c r="H14" s="2">
-        <v>0.7339</v>
-      </c>
-      <c r="I14" s="2">
-        <v>0.83160000000000001</v>
-      </c>
-      <c r="J14" s="2">
-        <v>0.70569999999999999</v>
+      <c r="D14" s="36">
+        <v>0.61450396615547298</v>
+      </c>
+      <c r="E14" s="36">
+        <v>0.55787234042553102</v>
+      </c>
+      <c r="F14" s="36">
+        <v>0.58108001265022102</v>
+      </c>
+      <c r="G14" s="36">
+        <v>0.63109318996415698</v>
+      </c>
+      <c r="H14" s="36">
+        <v>0.53144484553752902</v>
+      </c>
+      <c r="I14" s="36">
+        <v>0.606708742402992</v>
+      </c>
+      <c r="J14" s="36">
+        <v>0.52241679467485902</v>
       </c>
       <c r="K14" s="2"/>
-      <c r="W14" s="22"/>
+      <c r="W14" s="23"/>
       <c r="X14" s="25" t="s">
         <v>17</v>
       </c>
@@ -1405,137 +1439,137 @@
       </c>
       <c r="Z14">
         <f t="shared" si="1"/>
-        <v>0.84719999999999995</v>
-      </c>
-      <c r="AA14" s="35" t="s">
+        <v>0.63109318996415698</v>
+      </c>
+      <c r="AA14" s="20" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="15" spans="1:27" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="22"/>
-      <c r="B15" s="22"/>
+      <c r="A15" s="23"/>
+      <c r="B15" s="23"/>
       <c r="C15" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D15" s="2">
-        <v>0.95020000000000004</v>
-      </c>
-      <c r="E15" s="2">
-        <v>0.94650000000000001</v>
-      </c>
-      <c r="F15" s="2">
-        <v>0.94840000000000002</v>
-      </c>
-      <c r="G15" s="6">
-        <v>0.95040000000000002</v>
-      </c>
-      <c r="H15" s="2">
-        <v>0.94469999999999998</v>
-      </c>
-      <c r="I15" s="5">
-        <v>0.95579999999999998</v>
-      </c>
-      <c r="J15" s="2">
-        <v>0.88639999999999997</v>
+      <c r="D15" s="36">
+        <v>0.62380952380952304</v>
+      </c>
+      <c r="E15" s="36">
+        <v>0.621428571428571</v>
+      </c>
+      <c r="F15" s="36">
+        <v>0.62265306122448905</v>
+      </c>
+      <c r="G15" s="36">
+        <v>0.62397959183673402</v>
+      </c>
+      <c r="H15" s="36">
+        <v>0.62023809523809503</v>
+      </c>
+      <c r="I15" s="36">
+        <v>0.62755102040816302</v>
+      </c>
+      <c r="J15" s="36">
+        <v>0.58190476190476204</v>
       </c>
       <c r="K15" s="2"/>
-      <c r="W15" s="22"/>
-      <c r="X15" s="22"/>
+      <c r="W15" s="23"/>
+      <c r="X15" s="23"/>
       <c r="Y15" s="1" t="s">
         <v>15</v>
       </c>
       <c r="Z15">
         <f t="shared" si="1"/>
-        <v>0.95579999999999998</v>
-      </c>
-      <c r="AA15" s="35" t="s">
+        <v>0.62755102040816302</v>
+      </c>
+      <c r="AA15" s="20" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:27" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="31"/>
-      <c r="B16" s="31"/>
+      <c r="A16" s="26"/>
+      <c r="B16" s="26"/>
       <c r="C16" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="D16" s="16">
-        <v>0.94710000000000005</v>
-      </c>
-      <c r="E16" s="17">
-        <v>0.98470000000000002</v>
-      </c>
-      <c r="F16" s="16">
-        <v>0.96899999999999997</v>
-      </c>
-      <c r="G16" s="16">
-        <v>0.97150000000000003</v>
-      </c>
-      <c r="H16" s="16">
-        <v>0.96819999999999995</v>
-      </c>
-      <c r="I16" s="18">
-        <v>0.98729999999999996</v>
-      </c>
-      <c r="J16" s="16">
-        <v>0.93969999999999998</v>
-      </c>
-      <c r="K16" s="33"/>
-      <c r="W16" s="31"/>
-      <c r="X16" s="31"/>
+      <c r="D16" s="36">
+        <v>0.90191029138933099</v>
+      </c>
+      <c r="E16" s="36">
+        <v>0.94162331003351196</v>
+      </c>
+      <c r="F16" s="36">
+        <v>0.92568846208273403</v>
+      </c>
+      <c r="G16" s="36">
+        <v>0.92626003729736595</v>
+      </c>
+      <c r="H16" s="36">
+        <v>0.92319420734667501</v>
+      </c>
+      <c r="I16" s="36">
+        <v>0.94232125562658997</v>
+      </c>
+      <c r="J16" s="36">
+        <v>0.89758976475074304</v>
+      </c>
+      <c r="K16" s="2"/>
+      <c r="W16" s="26"/>
+      <c r="X16" s="26"/>
       <c r="Y16" s="15" t="s">
         <v>16</v>
       </c>
       <c r="Z16">
         <f t="shared" si="1"/>
-        <v>0.98729999999999996</v>
-      </c>
-      <c r="AA16" s="35" t="s">
+        <v>0.94232125562658997</v>
+      </c>
+      <c r="AA16" s="20" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="17" spans="1:28" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="18" spans="1:28" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="26" t="s">
+      <c r="A18" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B18" s="26" t="s">
+      <c r="B18" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="C18" s="28" t="s">
+      <c r="C18" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="D18" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E18" s="19" t="s">
-        <v>5</v>
-      </c>
-      <c r="F18" s="19" t="s">
-        <v>6</v>
-      </c>
-      <c r="G18" s="19" t="s">
-        <v>7</v>
-      </c>
-      <c r="H18" s="19" t="s">
-        <v>8</v>
-      </c>
-      <c r="I18" s="19" t="s">
-        <v>9</v>
-      </c>
-      <c r="J18" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="K18" s="33"/>
-      <c r="M18" s="26" t="s">
+      <c r="D18" t="s">
+        <v>29</v>
+      </c>
+      <c r="E18" t="s">
+        <v>30</v>
+      </c>
+      <c r="F18" t="s">
+        <v>31</v>
+      </c>
+      <c r="G18" t="s">
+        <v>32</v>
+      </c>
+      <c r="H18" t="s">
+        <v>33</v>
+      </c>
+      <c r="I18" t="s">
+        <v>34</v>
+      </c>
+      <c r="J18" t="s">
+        <v>35</v>
+      </c>
+      <c r="K18" s="2"/>
+      <c r="M18" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="N18" s="26" t="s">
+      <c r="N18" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="O18" s="28" t="s">
+      <c r="O18" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="P18" s="19" t="s">
+      <c r="P18" s="33" t="s">
         <v>5</v>
       </c>
       <c r="Q18" s="3" t="s">
@@ -1550,64 +1584,76 @@
       <c r="T18" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="U18" s="19" t="s">
+      <c r="U18" s="33" t="s">
         <v>6</v>
       </c>
       <c r="V18" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="Y18" s="26" t="s">
+      <c r="Y18" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="Z18" s="26" t="s">
+      <c r="Z18" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="AA18" s="28" t="s">
+      <c r="AA18" s="29" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="19" spans="1:28" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="27"/>
-      <c r="B19" s="27"/>
-      <c r="C19" s="29"/>
-      <c r="D19" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="E19" s="20"/>
-      <c r="F19" s="20"/>
-      <c r="G19" s="20"/>
-      <c r="H19" s="20"/>
-      <c r="I19" s="20"/>
-      <c r="J19" s="20"/>
-      <c r="K19" s="33"/>
-      <c r="M19" s="27"/>
-      <c r="N19" s="27"/>
-      <c r="O19" s="29"/>
-      <c r="P19" s="20"/>
+      <c r="A19" s="28"/>
+      <c r="B19" s="28"/>
+      <c r="C19" s="30"/>
+      <c r="D19" t="s">
+        <v>29</v>
+      </c>
+      <c r="E19" t="s">
+        <v>30</v>
+      </c>
+      <c r="F19" t="s">
+        <v>31</v>
+      </c>
+      <c r="G19" t="s">
+        <v>32</v>
+      </c>
+      <c r="H19" t="s">
+        <v>33</v>
+      </c>
+      <c r="I19" t="s">
+        <v>34</v>
+      </c>
+      <c r="J19" t="s">
+        <v>35</v>
+      </c>
+      <c r="K19" s="2"/>
+      <c r="M19" s="28"/>
+      <c r="N19" s="28"/>
+      <c r="O19" s="30"/>
+      <c r="P19" s="34"/>
       <c r="Q19" s="4"/>
       <c r="R19" s="4"/>
       <c r="S19" s="4"/>
       <c r="T19" s="4"/>
-      <c r="U19" s="20"/>
+      <c r="U19" s="34"/>
       <c r="V19" s="4" t="s">
         <v>4</v>
       </c>
       <c r="W19" t="s">
         <v>25</v>
       </c>
-      <c r="Y19" s="27"/>
-      <c r="Z19" s="27"/>
-      <c r="AA19" s="29"/>
+      <c r="Y19" s="28"/>
+      <c r="Z19" s="28"/>
+      <c r="AA19" s="30"/>
       <c r="AB19" t="str">
         <f>W19</f>
         <v>T-Test</v>
       </c>
     </row>
     <row r="20" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A20" s="21" t="s">
+      <c r="A20" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="B20" s="21" t="s">
+      <c r="B20" s="31" t="s">
         <v>12</v>
       </c>
       <c r="C20" s="1" t="s">
@@ -1623,29 +1669,29 @@
       </c>
       <c r="F20" s="2">
         <f t="shared" si="5"/>
+        <v>2</v>
+      </c>
+      <c r="G20" s="2">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="H20" s="2">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="I20" s="2">
+        <f t="shared" si="5"/>
+        <v>6</v>
+      </c>
+      <c r="J20" s="2">
+        <f t="shared" si="5"/>
         <v>3</v>
       </c>
-      <c r="G20" s="2">
-        <f t="shared" si="5"/>
-        <v>5</v>
-      </c>
-      <c r="H20" s="2">
-        <f t="shared" si="5"/>
-        <v>1</v>
-      </c>
-      <c r="I20" s="2">
-        <f t="shared" si="5"/>
-        <v>6</v>
-      </c>
-      <c r="J20" s="2">
-        <f t="shared" si="5"/>
-        <v>2</v>
-      </c>
       <c r="K20" s="2"/>
-      <c r="M20" s="21" t="s">
+      <c r="M20" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="N20" s="21" t="s">
+      <c r="N20" s="31" t="s">
         <v>12</v>
       </c>
       <c r="O20" s="1" t="s">
@@ -1676,23 +1722,23 @@
         <f>_xlfn.T.TEST(P20:T20,U20:V20,2,3)</f>
         <v>0.37637935813561824</v>
       </c>
-      <c r="Y20" s="21" t="s">
+      <c r="Y20" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="Z20" s="21" t="s">
+      <c r="Z20" s="31" t="s">
         <v>12</v>
       </c>
       <c r="AA20" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="AB20" s="34">
+      <c r="AB20" s="19">
         <f t="shared" ref="AB20:AB33" si="6">W20</f>
         <v>0.37637935813561824</v>
       </c>
     </row>
     <row r="21" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A21" s="22"/>
-      <c r="B21" s="22"/>
+      <c r="A21" s="23"/>
+      <c r="B21" s="23"/>
       <c r="C21" s="1" t="s">
         <v>14</v>
       </c>
@@ -1710,23 +1756,23 @@
       </c>
       <c r="G21" s="2">
         <f t="shared" si="5"/>
+        <v>4</v>
+      </c>
+      <c r="H21" s="2">
+        <f t="shared" si="5"/>
         <v>5</v>
       </c>
-      <c r="H21" s="2">
+      <c r="I21" s="2">
         <f t="shared" si="5"/>
         <v>3</v>
       </c>
-      <c r="I21" s="2">
-        <f t="shared" si="5"/>
-        <v>4</v>
-      </c>
       <c r="J21" s="2">
         <f t="shared" si="5"/>
         <v>7</v>
       </c>
       <c r="K21" s="2"/>
-      <c r="M21" s="22"/>
-      <c r="N21" s="22"/>
+      <c r="M21" s="23"/>
+      <c r="N21" s="23"/>
       <c r="O21" s="1" t="s">
         <v>14</v>
       </c>
@@ -1755,19 +1801,19 @@
         <f t="shared" ref="W21:W33" si="7">_xlfn.T.TEST(P21:T21,U21:V21,2,3)</f>
         <v>0.90674905801427308</v>
       </c>
-      <c r="Y21" s="22"/>
-      <c r="Z21" s="22"/>
+      <c r="Y21" s="23"/>
+      <c r="Z21" s="23"/>
       <c r="AA21" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="AB21" s="34">
+      <c r="AB21" s="19">
         <f>W21</f>
         <v>0.90674905801427308</v>
       </c>
     </row>
     <row r="22" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="22"/>
-      <c r="B22" s="22"/>
+      <c r="A22" s="23"/>
+      <c r="B22" s="23"/>
       <c r="C22" s="1" t="s">
         <v>15</v>
       </c>
@@ -1800,8 +1846,8 @@
         <v>7</v>
       </c>
       <c r="K22" s="2"/>
-      <c r="M22" s="22"/>
-      <c r="N22" s="22"/>
+      <c r="M22" s="23"/>
+      <c r="N22" s="23"/>
       <c r="O22" s="1" t="s">
         <v>15</v>
       </c>
@@ -1830,52 +1876,52 @@
         <f t="shared" si="7"/>
         <v>0.36128142129742197</v>
       </c>
-      <c r="Y22" s="22"/>
-      <c r="Z22" s="22"/>
+      <c r="Y22" s="23"/>
+      <c r="Z22" s="23"/>
       <c r="AA22" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="AB22" s="34">
+      <c r="AB22" s="19">
         <f t="shared" si="6"/>
         <v>0.36128142129742197</v>
       </c>
     </row>
     <row r="23" spans="1:28" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="22"/>
+      <c r="A23" s="23"/>
       <c r="B23" s="24"/>
       <c r="C23" s="7" t="s">
         <v>16</v>
       </c>
       <c r="D23" s="2">
         <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="E23" s="2">
+        <f t="shared" si="5"/>
+        <v>6</v>
+      </c>
+      <c r="F23" s="2">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="G23" s="2">
+        <f t="shared" si="5"/>
         <v>2</v>
       </c>
-      <c r="E23" s="2">
-        <f t="shared" si="5"/>
-        <v>6</v>
-      </c>
-      <c r="F23" s="2">
-        <f t="shared" si="5"/>
-        <v>5</v>
-      </c>
-      <c r="G23" s="2">
-        <f t="shared" si="5"/>
-        <v>1</v>
-      </c>
       <c r="H23" s="2">
         <f t="shared" si="5"/>
         <v>7</v>
       </c>
       <c r="I23" s="2">
         <f t="shared" si="5"/>
+        <v>3</v>
+      </c>
+      <c r="J23" s="2">
+        <f t="shared" si="5"/>
         <v>4</v>
       </c>
-      <c r="J23" s="2">
-        <f t="shared" si="5"/>
-        <v>3</v>
-      </c>
       <c r="K23" s="2"/>
-      <c r="M23" s="22"/>
+      <c r="M23" s="23"/>
       <c r="N23" s="24"/>
       <c r="O23" s="7" t="s">
         <v>16</v>
@@ -1905,18 +1951,18 @@
         <f t="shared" si="7"/>
         <v>0.54363106700340769</v>
       </c>
-      <c r="Y23" s="22"/>
+      <c r="Y23" s="23"/>
       <c r="Z23" s="24"/>
       <c r="AA23" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="AB23" s="34">
+      <c r="AB23" s="19">
         <f t="shared" si="6"/>
         <v>0.54363106700340769</v>
       </c>
     </row>
     <row r="24" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A24" s="22"/>
+      <c r="A24" s="23"/>
       <c r="B24" s="25" t="s">
         <v>17</v>
       </c>
@@ -1929,30 +1975,30 @@
       </c>
       <c r="E24" s="2">
         <f t="shared" si="5"/>
+        <v>3</v>
+      </c>
+      <c r="F24" s="2">
+        <f t="shared" si="5"/>
         <v>4</v>
       </c>
-      <c r="F24" s="2">
-        <f t="shared" si="5"/>
-        <v>3</v>
-      </c>
       <c r="G24" s="2">
         <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="H24" s="2">
+        <f t="shared" si="5"/>
+        <v>6</v>
+      </c>
+      <c r="I24" s="2">
+        <f t="shared" si="5"/>
+        <v>7</v>
+      </c>
+      <c r="J24" s="2">
+        <f t="shared" si="5"/>
         <v>2</v>
       </c>
-      <c r="H24" s="2">
-        <f t="shared" si="5"/>
-        <v>6</v>
-      </c>
-      <c r="I24" s="2">
-        <f t="shared" si="5"/>
-        <v>7</v>
-      </c>
-      <c r="J24" s="2">
-        <f t="shared" si="5"/>
-        <v>1</v>
-      </c>
       <c r="K24" s="2"/>
-      <c r="M24" s="22"/>
+      <c r="M24" s="23"/>
       <c r="N24" s="25" t="s">
         <v>17</v>
       </c>
@@ -1984,21 +2030,21 @@
         <f t="shared" si="7"/>
         <v>0.48586808144707244</v>
       </c>
-      <c r="Y24" s="22"/>
+      <c r="Y24" s="23"/>
       <c r="Z24" s="25" t="s">
         <v>17</v>
       </c>
       <c r="AA24" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="AB24" s="34">
+      <c r="AB24" s="19">
         <f t="shared" si="6"/>
         <v>0.48586808144707244</v>
       </c>
     </row>
     <row r="25" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A25" s="22"/>
-      <c r="B25" s="22"/>
+      <c r="A25" s="23"/>
+      <c r="B25" s="23"/>
       <c r="C25" s="1" t="s">
         <v>14</v>
       </c>
@@ -2008,12 +2054,12 @@
       </c>
       <c r="E25" s="2">
         <f t="shared" si="5"/>
+        <v>6</v>
+      </c>
+      <c r="F25" s="2">
+        <f t="shared" si="5"/>
         <v>7</v>
       </c>
-      <c r="F25" s="2">
-        <f t="shared" si="5"/>
-        <v>6</v>
-      </c>
       <c r="G25" s="2">
         <f t="shared" si="5"/>
         <v>1</v>
@@ -2031,8 +2077,8 @@
         <v>2</v>
       </c>
       <c r="K25" s="2"/>
-      <c r="M25" s="22"/>
-      <c r="N25" s="22"/>
+      <c r="M25" s="23"/>
+      <c r="N25" s="23"/>
       <c r="O25" s="1" t="s">
         <v>14</v>
       </c>
@@ -2061,19 +2107,19 @@
         <f t="shared" si="7"/>
         <v>0.83500141706692566</v>
       </c>
-      <c r="Y25" s="22"/>
-      <c r="Z25" s="22"/>
+      <c r="Y25" s="23"/>
+      <c r="Z25" s="23"/>
       <c r="AA25" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="AB25" s="34">
+      <c r="AB25" s="19">
         <f t="shared" si="6"/>
         <v>0.83500141706692566</v>
       </c>
     </row>
     <row r="26" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A26" s="22"/>
-      <c r="B26" s="22"/>
+      <c r="A26" s="23"/>
+      <c r="B26" s="23"/>
       <c r="C26" s="1" t="s">
         <v>15</v>
       </c>
@@ -2106,8 +2152,8 @@
         <v>5</v>
       </c>
       <c r="K26" s="2"/>
-      <c r="M26" s="22"/>
-      <c r="N26" s="22"/>
+      <c r="M26" s="23"/>
+      <c r="N26" s="23"/>
       <c r="O26" s="1" t="s">
         <v>15</v>
       </c>
@@ -2136,19 +2182,19 @@
         <f t="shared" si="7"/>
         <v>0.40994569453830498</v>
       </c>
-      <c r="Y26" s="22"/>
-      <c r="Z26" s="22"/>
+      <c r="Y26" s="23"/>
+      <c r="Z26" s="23"/>
       <c r="AA26" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="AB26" s="34">
+      <c r="AB26" s="19">
         <f t="shared" si="6"/>
         <v>0.40994569453830498</v>
       </c>
     </row>
     <row r="27" spans="1:28" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="23"/>
-      <c r="B27" s="23"/>
+      <c r="A27" s="32"/>
+      <c r="B27" s="32"/>
       <c r="C27" s="11" t="s">
         <v>16</v>
       </c>
@@ -2158,16 +2204,16 @@
       </c>
       <c r="E27" s="2">
         <f t="shared" si="5"/>
+        <v>2</v>
+      </c>
+      <c r="F27" s="2">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="G27" s="2">
+        <f t="shared" si="5"/>
         <v>3</v>
       </c>
-      <c r="F27" s="2">
-        <f t="shared" si="5"/>
-        <v>5</v>
-      </c>
-      <c r="G27" s="2">
-        <f t="shared" si="5"/>
-        <v>2</v>
-      </c>
       <c r="H27" s="2">
         <f t="shared" si="5"/>
         <v>6</v>
@@ -2181,8 +2227,8 @@
         <v>7</v>
       </c>
       <c r="K27" s="2"/>
-      <c r="M27" s="23"/>
-      <c r="N27" s="23"/>
+      <c r="M27" s="32"/>
+      <c r="N27" s="32"/>
       <c r="O27" s="11" t="s">
         <v>16</v>
       </c>
@@ -2211,21 +2257,21 @@
         <f t="shared" si="7"/>
         <v>0.92035361571434837</v>
       </c>
-      <c r="Y27" s="23"/>
-      <c r="Z27" s="23"/>
+      <c r="Y27" s="32"/>
+      <c r="Z27" s="32"/>
       <c r="AA27" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="AB27" s="34">
+      <c r="AB27" s="19">
         <f t="shared" si="6"/>
         <v>0.92035361571434837</v>
       </c>
     </row>
     <row r="28" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A28" s="30" t="s">
+      <c r="A28" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="B28" s="30" t="s">
+      <c r="B28" s="22" t="s">
         <v>12</v>
       </c>
       <c r="C28" s="1" t="s">
@@ -2233,37 +2279,37 @@
       </c>
       <c r="D28" s="2">
         <f t="shared" si="4"/>
+        <v>5</v>
+      </c>
+      <c r="E28" s="2">
+        <f t="shared" si="5"/>
+        <v>7</v>
+      </c>
+      <c r="F28" s="2">
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
-      <c r="E28" s="2">
-        <f t="shared" si="5"/>
-        <v>7</v>
-      </c>
-      <c r="F28" s="2">
+      <c r="G28" s="2">
+        <f t="shared" si="5"/>
+        <v>4</v>
+      </c>
+      <c r="H28" s="2">
+        <f t="shared" si="5"/>
+        <v>3</v>
+      </c>
+      <c r="I28" s="2">
+        <f t="shared" si="5"/>
+        <v>6</v>
+      </c>
+      <c r="J28" s="2">
         <f t="shared" si="5"/>
         <v>2</v>
       </c>
-      <c r="G28" s="2">
-        <f t="shared" si="5"/>
-        <v>3</v>
-      </c>
-      <c r="H28" s="2">
-        <f t="shared" si="5"/>
-        <v>5</v>
-      </c>
-      <c r="I28" s="2">
-        <f t="shared" si="5"/>
-        <v>6</v>
-      </c>
-      <c r="J28" s="2">
-        <f t="shared" si="5"/>
-        <v>4</v>
-      </c>
       <c r="K28" s="2"/>
-      <c r="M28" s="30" t="s">
+      <c r="M28" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="N28" s="30" t="s">
+      <c r="N28" s="22" t="s">
         <v>12</v>
       </c>
       <c r="O28" s="1" t="s">
@@ -2294,23 +2340,23 @@
         <f t="shared" si="7"/>
         <v>7.3378949092937726E-2</v>
       </c>
-      <c r="Y28" s="30" t="s">
+      <c r="Y28" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="Z28" s="30" t="s">
+      <c r="Z28" s="22" t="s">
         <v>12</v>
       </c>
       <c r="AA28" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="AB28" s="34">
+      <c r="AB28" s="19">
         <f t="shared" si="6"/>
         <v>7.3378949092937726E-2</v>
       </c>
     </row>
     <row r="29" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A29" s="22"/>
-      <c r="B29" s="22"/>
+      <c r="A29" s="23"/>
+      <c r="B29" s="23"/>
       <c r="C29" s="1" t="s">
         <v>15</v>
       </c>
@@ -2343,8 +2389,8 @@
         <v>6</v>
       </c>
       <c r="K29" s="2"/>
-      <c r="M29" s="22"/>
-      <c r="N29" s="22"/>
+      <c r="M29" s="23"/>
+      <c r="N29" s="23"/>
       <c r="O29" s="1" t="s">
         <v>15</v>
       </c>
@@ -2373,38 +2419,38 @@
         <f t="shared" si="7"/>
         <v>0.13493151129824396</v>
       </c>
-      <c r="Y29" s="22"/>
-      <c r="Z29" s="22"/>
+      <c r="Y29" s="23"/>
+      <c r="Z29" s="23"/>
       <c r="AA29" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="AB29" s="34">
+      <c r="AB29" s="19">
         <f t="shared" si="6"/>
         <v>0.13493151129824396</v>
       </c>
     </row>
     <row r="30" spans="1:28" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="22"/>
+      <c r="A30" s="23"/>
       <c r="B30" s="24"/>
       <c r="C30" s="7" t="s">
         <v>16</v>
       </c>
       <c r="D30" s="2">
         <f t="shared" si="4"/>
-        <v>6.5</v>
+        <v>6</v>
       </c>
       <c r="E30" s="2">
         <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="F30" s="2">
+        <f t="shared" si="5"/>
         <v>3</v>
       </c>
-      <c r="F30" s="2">
+      <c r="G30" s="2">
         <f t="shared" si="5"/>
         <v>2</v>
       </c>
-      <c r="G30" s="2">
-        <f t="shared" si="5"/>
-        <v>1</v>
-      </c>
       <c r="H30" s="2">
         <f t="shared" si="5"/>
         <v>4</v>
@@ -2415,10 +2461,10 @@
       </c>
       <c r="J30" s="2">
         <f t="shared" si="5"/>
-        <v>6.5</v>
+        <v>7</v>
       </c>
       <c r="K30" s="2"/>
-      <c r="M30" s="22"/>
+      <c r="M30" s="23"/>
       <c r="N30" s="24"/>
       <c r="O30" s="7" t="s">
         <v>16</v>
@@ -2448,18 +2494,18 @@
         <f t="shared" si="7"/>
         <v>0.75694751563673712</v>
       </c>
-      <c r="Y30" s="22"/>
+      <c r="Y30" s="23"/>
       <c r="Z30" s="24"/>
       <c r="AA30" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="AB30" s="34">
+      <c r="AB30" s="19">
         <f t="shared" si="6"/>
         <v>0.75694751563673712</v>
       </c>
     </row>
     <row r="31" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A31" s="22"/>
+      <c r="A31" s="23"/>
       <c r="B31" s="25" t="s">
         <v>17</v>
       </c>
@@ -2495,7 +2541,7 @@
         <v>7</v>
       </c>
       <c r="K31" s="2"/>
-      <c r="M31" s="22"/>
+      <c r="M31" s="23"/>
       <c r="N31" s="25" t="s">
         <v>17</v>
       </c>
@@ -2527,21 +2573,21 @@
         <f t="shared" si="7"/>
         <v>0.37857042761468757</v>
       </c>
-      <c r="Y31" s="22"/>
+      <c r="Y31" s="23"/>
       <c r="Z31" s="25" t="s">
         <v>17</v>
       </c>
       <c r="AA31" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="AB31" s="34">
+      <c r="AB31" s="19">
         <f t="shared" si="6"/>
         <v>0.37857042761468757</v>
       </c>
     </row>
     <row r="32" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A32" s="22"/>
-      <c r="B32" s="22"/>
+      <c r="A32" s="23"/>
+      <c r="B32" s="23"/>
       <c r="C32" s="1" t="s">
         <v>15</v>
       </c>
@@ -2574,8 +2620,8 @@
         <v>7</v>
       </c>
       <c r="K32" s="2"/>
-      <c r="M32" s="22"/>
-      <c r="N32" s="22"/>
+      <c r="M32" s="23"/>
+      <c r="N32" s="23"/>
       <c r="O32" s="1" t="s">
         <v>15</v>
       </c>
@@ -2604,19 +2650,19 @@
         <f t="shared" si="7"/>
         <v>0.38102067341463308</v>
       </c>
-      <c r="Y32" s="22"/>
-      <c r="Z32" s="22"/>
+      <c r="Y32" s="23"/>
+      <c r="Z32" s="23"/>
       <c r="AA32" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="AB32" s="34">
+      <c r="AB32" s="19">
         <f t="shared" si="6"/>
         <v>0.38102067341463308</v>
       </c>
     </row>
     <row r="33" spans="1:28" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="31"/>
-      <c r="B33" s="31"/>
+      <c r="A33" s="26"/>
+      <c r="B33" s="26"/>
       <c r="C33" s="15" t="s">
         <v>16</v>
       </c>
@@ -2649,8 +2695,8 @@
         <v>7</v>
       </c>
       <c r="K33" s="2"/>
-      <c r="M33" s="31"/>
-      <c r="N33" s="31"/>
+      <c r="M33" s="26"/>
+      <c r="N33" s="26"/>
       <c r="O33" s="15" t="s">
         <v>16</v>
       </c>
@@ -2679,12 +2725,12 @@
         <f t="shared" si="7"/>
         <v>0.45821287679844458</v>
       </c>
-      <c r="Y33" s="31"/>
-      <c r="Z33" s="31"/>
+      <c r="Y33" s="26"/>
+      <c r="Z33" s="26"/>
       <c r="AA33" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="AB33" s="34">
+      <c r="AB33" s="19">
         <f t="shared" si="6"/>
         <v>0.45821287679844458</v>
       </c>
@@ -2695,19 +2741,19 @@
       </c>
       <c r="D34" s="2">
         <f>AVERAGE(D20:D33)</f>
-        <v>3.6428571428571428</v>
+        <v>3.8214285714285716</v>
       </c>
       <c r="E34" s="2">
         <f t="shared" ref="E34:J34" si="8">AVERAGE(E20:E33)</f>
-        <v>4.0714285714285712</v>
+        <v>3.7142857142857144</v>
       </c>
       <c r="F34" s="2">
         <f t="shared" si="8"/>
-        <v>4.1785714285714288</v>
+        <v>4.25</v>
       </c>
       <c r="G34" s="2">
         <f t="shared" si="8"/>
-        <v>2.9285714285714284</v>
+        <v>3.0714285714285716</v>
       </c>
       <c r="H34" s="2">
         <f t="shared" si="8"/>
@@ -2715,11 +2761,11 @@
       </c>
       <c r="I34" s="2">
         <f t="shared" si="8"/>
-        <v>3.5714285714285716</v>
+        <v>3.4285714285714284</v>
       </c>
       <c r="J34" s="2">
         <f t="shared" si="8"/>
-        <v>5.1071428571428568</v>
+        <v>5.2142857142857144</v>
       </c>
       <c r="K34" s="2"/>
     </row>
@@ -2729,11 +2775,11 @@
       </c>
       <c r="D35" s="2">
         <f>_xlfn.RANK.AVG(D34, $D34:$J34, 1)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E35" s="2">
         <f t="shared" ref="E35:J35" si="9">_xlfn.RANK.AVG(E34, $D34:$J34, 1)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F35" s="2">
         <f t="shared" si="9"/>
@@ -2758,22 +2804,30 @@
       <c r="K35" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="58">
-    <mergeCell ref="X11:X13"/>
-    <mergeCell ref="X14:X16"/>
-    <mergeCell ref="W1:W2"/>
-    <mergeCell ref="X1:X2"/>
-    <mergeCell ref="Y1:Y2"/>
-    <mergeCell ref="W3:W10"/>
-    <mergeCell ref="X3:X6"/>
-    <mergeCell ref="X7:X10"/>
-    <mergeCell ref="AA18:AA19"/>
-    <mergeCell ref="Y20:Y27"/>
-    <mergeCell ref="Z20:Z23"/>
-    <mergeCell ref="Z24:Z27"/>
-    <mergeCell ref="Y28:Y33"/>
-    <mergeCell ref="Z28:Z30"/>
-    <mergeCell ref="Z31:Z33"/>
+  <mergeCells count="52">
+    <mergeCell ref="A3:A10"/>
+    <mergeCell ref="B3:B6"/>
+    <mergeCell ref="B7:B10"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="A11:A16"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="A20:A27"/>
+    <mergeCell ref="B20:B23"/>
+    <mergeCell ref="B24:B27"/>
+    <mergeCell ref="A28:A33"/>
+    <mergeCell ref="B28:B30"/>
+    <mergeCell ref="B31:B33"/>
+    <mergeCell ref="M3:M6"/>
+    <mergeCell ref="M7:M9"/>
+    <mergeCell ref="Q3:Q5"/>
+    <mergeCell ref="Q6:Q8"/>
+    <mergeCell ref="V3:V4"/>
+    <mergeCell ref="V5:V6"/>
     <mergeCell ref="M28:M33"/>
     <mergeCell ref="N28:N30"/>
     <mergeCell ref="N31:N33"/>
@@ -2787,36 +2841,22 @@
     <mergeCell ref="O18:O19"/>
     <mergeCell ref="P18:P19"/>
     <mergeCell ref="U18:U19"/>
+    <mergeCell ref="AA18:AA19"/>
+    <mergeCell ref="Y20:Y27"/>
+    <mergeCell ref="Z20:Z23"/>
+    <mergeCell ref="Z24:Z27"/>
+    <mergeCell ref="Y28:Y33"/>
+    <mergeCell ref="Z28:Z30"/>
+    <mergeCell ref="Z31:Z33"/>
+    <mergeCell ref="X11:X13"/>
+    <mergeCell ref="X14:X16"/>
+    <mergeCell ref="W1:W2"/>
+    <mergeCell ref="X1:X2"/>
+    <mergeCell ref="Y1:Y2"/>
+    <mergeCell ref="W3:W10"/>
+    <mergeCell ref="X3:X6"/>
+    <mergeCell ref="X7:X10"/>
     <mergeCell ref="W11:W16"/>
-    <mergeCell ref="M3:M6"/>
-    <mergeCell ref="M7:M9"/>
-    <mergeCell ref="Q3:Q5"/>
-    <mergeCell ref="Q6:Q8"/>
-    <mergeCell ref="V3:V4"/>
-    <mergeCell ref="V5:V6"/>
-    <mergeCell ref="A20:A27"/>
-    <mergeCell ref="B20:B23"/>
-    <mergeCell ref="B24:B27"/>
-    <mergeCell ref="A28:A33"/>
-    <mergeCell ref="B28:B30"/>
-    <mergeCell ref="B31:B33"/>
-    <mergeCell ref="J18:J19"/>
-    <mergeCell ref="A11:A16"/>
-    <mergeCell ref="B11:B13"/>
-    <mergeCell ref="B14:B16"/>
-    <mergeCell ref="A18:A19"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="E18:E19"/>
-    <mergeCell ref="F18:F19"/>
-    <mergeCell ref="G18:G19"/>
-    <mergeCell ref="H18:H19"/>
-    <mergeCell ref="I18:I19"/>
-    <mergeCell ref="A3:A10"/>
-    <mergeCell ref="B3:B6"/>
-    <mergeCell ref="B7:B10"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>